<commit_message>
Format correction for files
</commit_message>
<xml_diff>
--- a/InputData/add-outputs/NoH/Number of Households.xlsx
+++ b/InputData/add-outputs/NoH/Number of Households.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\내 드라이브\2026\01.EPS\05.EPS고도화\01.EPS 4.0.5 update\v4.0.5\add-outputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-southkorea\InputData\add-outputs\NoH\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{063B4943-9203-43ED-822B-4C56063659EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6332807-A7DE-4256-BC67-BD1DF25FE3B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -269,11 +269,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -281,21 +281,21 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="18"/>
       <color theme="3"/>
-      <name val="맑은 고딕"/>
+      <name val="Cambria"/>
       <family val="2"/>
       <scheme val="major"/>
     </font>
@@ -303,7 +303,7 @@
       <b/>
       <sz val="15"/>
       <color theme="3"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -311,7 +311,7 @@
       <b/>
       <sz val="13"/>
       <color theme="3"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -319,28 +319,28 @@
       <b/>
       <sz val="11"/>
       <color theme="3"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -348,7 +348,7 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -356,14 +356,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -371,14 +371,14 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -386,14 +386,14 @@
       <i/>
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -420,13 +420,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -434,14 +434,14 @@
     <font>
       <sz val="11"/>
       <color indexed="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -954,9 +954,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="22" fillId="34" borderId="14" xfId="74" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
@@ -976,31 +973,44 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="75">
-    <cellStyle name="20% - 강조색1" xfId="18" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색2" xfId="21" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색3" xfId="24" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색4" xfId="27" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색5" xfId="30" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색6" xfId="33" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색1" xfId="19" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색2" xfId="22" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색3" xfId="25" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색4" xfId="28" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색5" xfId="31" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색6" xfId="34" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="20% - Accent1" xfId="18" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="21" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="24" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="27" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="30" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="33" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="19" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="22" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="25" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="28" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="31" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="34" builtinId="51" customBuiltin="1"/>
     <cellStyle name="60% - Accent1 2" xfId="62" xr:uid="{7D4913BE-1660-475B-88D4-714E8A641CFB}"/>
     <cellStyle name="60% - Accent2 2" xfId="63" xr:uid="{E18DA92F-95CC-4882-BBE6-08084463355B}"/>
     <cellStyle name="60% - Accent3 2" xfId="64" xr:uid="{3D7AA9D9-39BB-404D-82B7-1179141C06D3}"/>
     <cellStyle name="60% - Accent4 2" xfId="65" xr:uid="{AB77D1E1-0C03-48A6-82C6-F8C803DAB0D4}"/>
     <cellStyle name="60% - Accent5 2" xfId="66" xr:uid="{741B7963-9D58-462B-9B00-F2AFEE0DEE08}"/>
     <cellStyle name="60% - Accent6 2" xfId="67" xr:uid="{D898A326-A2CF-46B5-815E-CCFFA4AA3BA6}"/>
+    <cellStyle name="Accent1" xfId="17" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="20" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="23" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="26" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="29" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="32" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Body: normal cell" xfId="36" xr:uid="{EA3F03DA-DAAC-4E67-9C48-32345E5792CA}"/>
     <cellStyle name="Body: normal cell 2" xfId="52" xr:uid="{08CD34FB-32D1-4D4E-B78E-6D9F0921375F}"/>
     <cellStyle name="Body: normal cell 3" xfId="44" xr:uid="{3455BC5E-F6FE-45B4-B515-07C1FF8A7B97}"/>
     <cellStyle name="Body: normal cell 4" xfId="68" xr:uid="{235B8F88-29E6-46ED-B2CB-1EE68DFFBB5C}"/>
+    <cellStyle name="Calculation" xfId="10" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="12" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="15" builtinId="53" customBuiltin="1"/>
     <cellStyle name="Font: Calibri, 9pt regular" xfId="37" xr:uid="{046FC022-7ADB-439F-AC6B-06F1FB0969A9}"/>
     <cellStyle name="Font: Calibri, 9pt regular 2" xfId="53" xr:uid="{F67B9D4D-81FC-422B-BE16-8FCFA80B6324}"/>
     <cellStyle name="Font: Calibri, 9pt regular 3" xfId="45" xr:uid="{B9AB311C-4622-44DC-95B7-A3EE560BED6E}"/>
@@ -1009,11 +1019,19 @@
     <cellStyle name="Footnotes: top row 2" xfId="54" xr:uid="{FAE885D7-0ED1-4F57-9C86-3E57F5B776CA}"/>
     <cellStyle name="Footnotes: top row 3" xfId="46" xr:uid="{6D3A535B-FE51-41C9-A1AF-6CC2E6D28C13}"/>
     <cellStyle name="Footnotes: top row 4" xfId="70" xr:uid="{D55444D5-5FDB-452E-9A25-4FBC5024891F}"/>
+    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
     <cellStyle name="Header: bottom row" xfId="39" xr:uid="{1B3E9918-1BEB-4E26-9226-DDCFB4A4D031}"/>
     <cellStyle name="Header: bottom row 2" xfId="55" xr:uid="{4F80F3A6-0CFF-4FA5-96E2-ADE6F1F6B9E1}"/>
     <cellStyle name="Header: bottom row 3" xfId="47" xr:uid="{99198BBE-FF67-47E8-8D1B-44FF5F9DAF26}"/>
     <cellStyle name="Header: bottom row 4" xfId="71" xr:uid="{97A7D3E4-344A-41A0-A4B7-78E77DCD1453}"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="8" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="11" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral 2" xfId="61" xr:uid="{9752847A-6ACD-42F9-AFB4-C2A2E9213018}"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="51" xr:uid="{2F0F7E80-8BCA-4A78-8B67-35323ECD9B42}"/>
     <cellStyle name="Normal 3" xfId="50" xr:uid="{60154007-A150-4910-8900-986DA2B8C17E}"/>
     <cellStyle name="Normal 3 2" xfId="59" xr:uid="{7C665A8E-D301-430C-9E6F-6F85D41847C9}"/>
@@ -1022,6 +1040,8 @@
     <cellStyle name="Normal 5 2" xfId="60" xr:uid="{801F20AC-8EC6-4D23-972B-E25ECAB445C9}"/>
     <cellStyle name="Normal 6" xfId="58" xr:uid="{963376A2-6DCB-443C-B7BC-658DC602F929}"/>
     <cellStyle name="Normal 7" xfId="35" xr:uid="{6F59A552-82E2-4373-88A6-95B1E6D451CC}"/>
+    <cellStyle name="Note" xfId="14" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="9" builtinId="21" customBuiltin="1"/>
     <cellStyle name="Parent row" xfId="40" xr:uid="{BB70FD24-CC8A-4059-A8FB-EF3473AEE5BF}"/>
     <cellStyle name="Parent row 2" xfId="56" xr:uid="{E64DB29F-0F99-4575-888E-643D4F638507}"/>
     <cellStyle name="Parent row 3" xfId="48" xr:uid="{E7854F2A-5513-4980-9AA1-ADA6421310AC}"/>
@@ -1030,29 +1050,9 @@
     <cellStyle name="Table title 2" xfId="57" xr:uid="{B08EF0C1-BB7F-43EF-93CB-237A779E958C}"/>
     <cellStyle name="Table title 3" xfId="49" xr:uid="{AB3CAFA1-44B0-47FC-9653-B91E22DB566D}"/>
     <cellStyle name="Table title 4" xfId="73" xr:uid="{DB43BB74-3283-438D-B986-0BAB8FC15190}"/>
-    <cellStyle name="강조색1" xfId="17" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="강조색2" xfId="20" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="강조색3" xfId="23" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="강조색4" xfId="26" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="강조색5" xfId="29" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="강조색6" xfId="32" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="경고문" xfId="13" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="계산" xfId="10" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="나쁨" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="메모" xfId="14" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="설명 텍스트" xfId="15" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="셀 확인" xfId="12" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="연결된 셀" xfId="11" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="요약" xfId="16" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="입력" xfId="8" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="제목" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="제목 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="제목 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="제목 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="제목 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="좋음" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="출력" xfId="9" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Total" xfId="16" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="13" builtinId="11" customBuiltin="1"/>
     <cellStyle name="표준 2" xfId="74" xr:uid="{FC4CE50F-F1FC-43E8-8B43-8D39CDFDA6B8}"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1378,70 +1378,70 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="38.25" customWidth="1"/>
+    <col min="2" max="2" width="38.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2">
       <c r="B4" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2">
       <c r="B5" s="2">
         <v>2026</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2">
       <c r="B6" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2">
       <c r="B7" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B9" s="4">
+    <row r="9" spans="1:2">
+      <c r="B9" s="3">
         <v>2021</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2">
       <c r="B10" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2">
       <c r="B11" s="2">
         <v>2026</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2">
       <c r="B12" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2">
       <c r="B13" s="2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2">
       <c r="B14" s="2"/>
     </row>
   </sheetData>
@@ -1454,536 +1454,536 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58377776-1A7D-4F38-88D4-5A6404236C90}">
   <dimension ref="A1:AI17"/>
-  <sheetFormatPr defaultColWidth="21" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="21" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="16384" width="21" style="7"/>
+    <col min="1" max="16384" width="21" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:35" ht="20.149999999999999" customHeight="1">
+      <c r="A1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="N1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="O1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="P1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="Q1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="R1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="S1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="T1" s="6" t="s">
+      <c r="T1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="U1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="V1" s="6" t="s">
+      <c r="V1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="W1" s="6" t="s">
+      <c r="W1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="X1" s="6" t="s">
+      <c r="X1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="Y1" s="6" t="s">
+      <c r="Y1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="Z1" s="6" t="s">
+      <c r="Z1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="AA1" s="6" t="s">
+      <c r="AA1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="AB1" s="6" t="s">
+      <c r="AB1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AC1" s="6" t="s">
+      <c r="AC1" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="AD1" s="6" t="s">
+      <c r="AD1" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="AE1" s="6" t="s">
+      <c r="AE1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AF1" s="6" t="s">
+      <c r="AF1" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="AG1" s="6" t="s">
+      <c r="AG1" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="AH1" s="6" t="s">
+      <c r="AH1" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="AI1" s="6" t="s">
+      <c r="AI1" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:35" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
+    <row r="2" spans="1:35" ht="20.149999999999999" customHeight="1">
+      <c r="A2" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="8">
         <v>20730614</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="8">
         <v>21272581</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="8">
         <v>21663978</v>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="8">
         <v>21970523</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="8">
         <v>22179969</v>
       </c>
-      <c r="H2" s="9">
+      <c r="H2" s="8">
         <v>22388821</v>
       </c>
-      <c r="I2" s="9">
+      <c r="I2" s="8">
         <v>22597677</v>
       </c>
-      <c r="J2" s="9">
+      <c r="J2" s="8">
         <v>22806529</v>
       </c>
-      <c r="K2" s="9">
+      <c r="K2" s="8">
         <v>23000187</v>
       </c>
-      <c r="L2" s="9">
+      <c r="L2" s="8">
         <v>23180688</v>
       </c>
-      <c r="M2" s="9">
+      <c r="M2" s="8">
         <v>23348528</v>
       </c>
-      <c r="N2" s="9">
+      <c r="N2" s="8">
         <v>23506021</v>
       </c>
-      <c r="O2" s="9">
+      <c r="O2" s="8">
         <v>23651567</v>
       </c>
-      <c r="P2" s="9">
+      <c r="P2" s="8">
         <v>23786407</v>
       </c>
-      <c r="Q2" s="9">
+      <c r="Q2" s="8">
         <v>23908631</v>
       </c>
-      <c r="R2" s="9">
+      <c r="R2" s="8">
         <v>24019901</v>
       </c>
-      <c r="S2" s="9">
+      <c r="S2" s="8">
         <v>24119593</v>
       </c>
-      <c r="T2" s="9">
+      <c r="T2" s="8">
         <v>24204775</v>
       </c>
-      <c r="U2" s="9">
+      <c r="U2" s="8">
         <v>24273745</v>
       </c>
-      <c r="V2" s="9">
+      <c r="V2" s="8">
         <v>24325345</v>
       </c>
-      <c r="W2" s="9">
+      <c r="W2" s="8">
         <v>24358286</v>
       </c>
-      <c r="X2" s="9">
+      <c r="X2" s="8">
         <v>24371931</v>
       </c>
-      <c r="Y2" s="9">
+      <c r="Y2" s="8">
         <v>24365630</v>
       </c>
-      <c r="Z2" s="9">
+      <c r="Z2" s="8">
         <v>24338645</v>
       </c>
-      <c r="AA2" s="9">
+      <c r="AA2" s="8">
         <v>24290684</v>
       </c>
-      <c r="AB2" s="9">
+      <c r="AB2" s="8">
         <v>24221145</v>
       </c>
-      <c r="AC2" s="9">
+      <c r="AC2" s="8">
         <v>24131623</v>
       </c>
-      <c r="AD2" s="9">
+      <c r="AD2" s="8">
         <v>24023713</v>
       </c>
-      <c r="AE2" s="9">
+      <c r="AE2" s="8">
         <v>23899146</v>
       </c>
-      <c r="AF2" s="9">
+      <c r="AF2" s="8">
         <v>23760443</v>
       </c>
-      <c r="AG2" s="9">
+      <c r="AG2" s="8">
         <v>23609533</v>
       </c>
-      <c r="AH2" s="9">
+      <c r="AH2" s="8">
         <v>23447961</v>
       </c>
-      <c r="AI2" s="9">
+      <c r="AI2" s="8">
         <v>23277470</v>
       </c>
     </row>
-    <row r="3" spans="1:35" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
+    <row r="3" spans="1:35" ht="20.149999999999999" customHeight="1">
+      <c r="A3" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="8">
         <v>14009289</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="8">
         <v>14192205</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="8">
         <v>14313314</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="8">
         <v>14413852</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G3" s="8">
         <v>14455067</v>
       </c>
-      <c r="H3" s="9">
+      <c r="H3" s="8">
         <v>14496150</v>
       </c>
-      <c r="I3" s="9">
+      <c r="I3" s="8">
         <v>14537244</v>
       </c>
-      <c r="J3" s="9">
+      <c r="J3" s="8">
         <v>14578324</v>
       </c>
-      <c r="K3" s="9">
+      <c r="K3" s="8">
         <v>14619343</v>
       </c>
-      <c r="L3" s="9">
+      <c r="L3" s="8">
         <v>14655309</v>
       </c>
-      <c r="M3" s="9">
+      <c r="M3" s="8">
         <v>14685834</v>
       </c>
-      <c r="N3" s="9">
+      <c r="N3" s="8">
         <v>14710683</v>
       </c>
-      <c r="O3" s="9">
+      <c r="O3" s="8">
         <v>14729719</v>
       </c>
-      <c r="P3" s="9">
+      <c r="P3" s="8">
         <v>14743899</v>
       </c>
-      <c r="Q3" s="9">
+      <c r="Q3" s="8">
         <v>14753391</v>
       </c>
-      <c r="R3" s="9">
+      <c r="R3" s="8">
         <v>14758309</v>
       </c>
-      <c r="S3" s="9">
+      <c r="S3" s="8">
         <v>14758526</v>
       </c>
-      <c r="T3" s="9">
+      <c r="T3" s="8">
         <v>14753119</v>
       </c>
-      <c r="U3" s="9">
+      <c r="U3" s="8">
         <v>14740922</v>
       </c>
-      <c r="V3" s="9">
+      <c r="V3" s="8">
         <v>14721363</v>
       </c>
-      <c r="W3" s="9">
+      <c r="W3" s="8">
         <v>14693440</v>
       </c>
-      <c r="X3" s="9">
+      <c r="X3" s="8">
         <v>14656554</v>
       </c>
-      <c r="Y3" s="9">
+      <c r="Y3" s="8">
         <v>14610054</v>
       </c>
-      <c r="Z3" s="9">
+      <c r="Z3" s="8">
         <v>14553734</v>
       </c>
-      <c r="AA3" s="9">
+      <c r="AA3" s="8">
         <v>14487297</v>
       </c>
-      <c r="AB3" s="9">
+      <c r="AB3" s="8">
         <v>14410259</v>
       </c>
-      <c r="AC3" s="9">
+      <c r="AC3" s="8">
         <v>14323010</v>
       </c>
-      <c r="AD3" s="9">
+      <c r="AD3" s="8">
         <v>14225553</v>
       </c>
-      <c r="AE3" s="9">
+      <c r="AE3" s="8">
         <v>14118838</v>
       </c>
-      <c r="AF3" s="9">
+      <c r="AF3" s="8">
         <v>14004024</v>
       </c>
-      <c r="AG3" s="9">
+      <c r="AG3" s="8">
         <v>13881810</v>
       </c>
-      <c r="AH3" s="9">
+      <c r="AH3" s="8">
         <v>13753528</v>
       </c>
-      <c r="AI3" s="9">
+      <c r="AI3" s="8">
         <v>13620879</v>
       </c>
     </row>
-    <row r="4" spans="1:35" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:35" ht="20.149999999999999" customHeight="1">
+      <c r="A4" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C4" s="8">
         <v>6721325</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="8">
         <v>7080376</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="8">
         <v>7350664</v>
       </c>
-      <c r="F4" s="9">
+      <c r="F4" s="8">
         <v>7556671</v>
       </c>
-      <c r="G4" s="9">
+      <c r="G4" s="8">
         <v>7724902</v>
       </c>
-      <c r="H4" s="9">
+      <c r="H4" s="8">
         <v>7892671</v>
       </c>
-      <c r="I4" s="9">
+      <c r="I4" s="8">
         <v>8060433</v>
       </c>
-      <c r="J4" s="9">
+      <c r="J4" s="8">
         <v>8228205</v>
       </c>
-      <c r="K4" s="9">
+      <c r="K4" s="8">
         <v>8380844</v>
       </c>
-      <c r="L4" s="9">
+      <c r="L4" s="8">
         <v>8525379</v>
       </c>
-      <c r="M4" s="9">
+      <c r="M4" s="8">
         <v>8662694</v>
       </c>
-      <c r="N4" s="9">
+      <c r="N4" s="8">
         <v>8795338</v>
       </c>
-      <c r="O4" s="9">
+      <c r="O4" s="8">
         <v>8921848</v>
       </c>
-      <c r="P4" s="9">
+      <c r="P4" s="8">
         <v>9042508</v>
       </c>
-      <c r="Q4" s="9">
+      <c r="Q4" s="8">
         <v>9155240</v>
       </c>
-      <c r="R4" s="9">
+      <c r="R4" s="8">
         <v>9261592</v>
       </c>
-      <c r="S4" s="9">
+      <c r="S4" s="8">
         <v>9361067</v>
       </c>
-      <c r="T4" s="9">
+      <c r="T4" s="8">
         <v>9451656</v>
       </c>
-      <c r="U4" s="9">
+      <c r="U4" s="8">
         <v>9532823</v>
       </c>
-      <c r="V4" s="9">
+      <c r="V4" s="8">
         <v>9603982</v>
       </c>
-      <c r="W4" s="9">
+      <c r="W4" s="8">
         <v>9664846</v>
       </c>
-      <c r="X4" s="9">
+      <c r="X4" s="8">
         <v>9715377</v>
       </c>
-      <c r="Y4" s="9">
+      <c r="Y4" s="8">
         <v>9755576</v>
       </c>
-      <c r="Z4" s="9">
+      <c r="Z4" s="8">
         <v>9784911</v>
       </c>
-      <c r="AA4" s="9">
+      <c r="AA4" s="8">
         <v>9803387</v>
       </c>
-      <c r="AB4" s="9">
+      <c r="AB4" s="8">
         <v>9810886</v>
       </c>
-      <c r="AC4" s="9">
+      <c r="AC4" s="8">
         <v>9808613</v>
       </c>
-      <c r="AD4" s="9">
+      <c r="AD4" s="8">
         <v>9798160</v>
       </c>
-      <c r="AE4" s="9">
+      <c r="AE4" s="8">
         <v>9780308</v>
       </c>
-      <c r="AF4" s="9">
+      <c r="AF4" s="8">
         <v>9756419</v>
       </c>
-      <c r="AG4" s="9">
+      <c r="AG4" s="8">
         <v>9727723</v>
       </c>
-      <c r="AH4" s="9">
+      <c r="AH4" s="8">
         <v>9694433</v>
       </c>
-      <c r="AI4" s="9">
+      <c r="AI4" s="8">
         <v>9656591</v>
       </c>
     </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A8" s="11" t="s">
+    <row r="8" spans="1:35">
+      <c r="A8" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-    </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A9" s="11" t="s">
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+    </row>
+    <row r="9" spans="1:35">
+      <c r="A9" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-    </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A10" s="11" t="s">
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+    </row>
+    <row r="10" spans="1:35">
+      <c r="A10" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-    </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A11" s="11" t="s">
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+    </row>
+    <row r="11" spans="1:35">
+      <c r="A11" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-    </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A12" s="11" t="s">
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+    </row>
+    <row r="12" spans="1:35">
+      <c r="A12" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-    </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A13" s="11" t="s">
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+    </row>
+    <row r="13" spans="1:35">
+      <c r="A13" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-    </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A14" s="11" t="s">
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+    </row>
+    <row r="14" spans="1:35">
+      <c r="A14" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-    </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A15" s="11" t="s">
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+    </row>
+    <row r="15" spans="1:35">
+      <c r="A15" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B15" s="12"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-    </row>
-    <row r="16" spans="1:35" x14ac:dyDescent="0.2">
-      <c r="A16" s="11" t="s">
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+    </row>
+    <row r="16" spans="1:35">
+      <c r="A16" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="11" t="s">
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="21" type="noConversion"/>
@@ -1994,162 +1994,162 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDBBA753-B79C-4865-AC77-3F085ACCA0CD}">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultColWidth="21" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="21" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="16384" width="21" style="7"/>
+    <col min="1" max="16384" width="21" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:7" ht="20.149999999999999" customHeight="1">
+      <c r="A1" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+    <row r="2" spans="1:7" ht="20.149999999999999" customHeight="1">
+      <c r="A2" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="8">
         <v>23093108</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="8">
         <v>23472895</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="8">
         <v>23705814</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="8">
         <v>23914851</v>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="8">
         <v>24118928</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="8">
         <v>24300087</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="11" t="s">
+    <row r="6" spans="1:7">
+      <c r="A6" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="12"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="11" t="s">
+      <c r="C6" s="11"/>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="12"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="11" t="s">
+      <c r="C7" s="11"/>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="12"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="11" t="s">
+      <c r="C8" s="11"/>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="12"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="11" t="s">
+      <c r="C9" s="11"/>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C10" s="12"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="11" t="s">
+      <c r="C10" s="11"/>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C11" s="12"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="11" t="s">
+      <c r="C11" s="11"/>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C12" s="12"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="11" t="s">
+      <c r="C12" s="11"/>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="C13" s="12"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="11" t="s">
+      <c r="C13" s="11"/>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="11" t="s">
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="C15" s="12"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="11" t="s">
+      <c r="C15" s="11"/>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="12"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="11" t="s">
+      <c r="C16" s="11"/>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C17" s="12"/>
+      <c r="C17" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="21" type="noConversion"/>
@@ -2163,229 +2163,230 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE2"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="2" width="16.5" customWidth="1"/>
-    <col min="3" max="3" width="9.875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="16.453125" style="12" customWidth="1"/>
+    <col min="3" max="3" width="9.90625" style="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.26953125" style="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.7265625" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:31">
+      <c r="A1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="3">
+      <c r="B1" s="13">
         <v>2021</v>
       </c>
-      <c r="C1" s="3">
+      <c r="C1" s="13">
         <v>2022</v>
       </c>
-      <c r="D1" s="3">
+      <c r="D1" s="13">
         <v>2023</v>
       </c>
-      <c r="E1" s="3">
+      <c r="E1" s="13">
         <v>2024</v>
       </c>
-      <c r="F1" s="3">
+      <c r="F1" s="13">
         <v>2025</v>
       </c>
-      <c r="G1" s="3">
+      <c r="G1" s="13">
         <v>2026</v>
       </c>
-      <c r="H1" s="3">
+      <c r="H1" s="13">
         <v>2027</v>
       </c>
-      <c r="I1" s="3">
+      <c r="I1" s="13">
         <v>2028</v>
       </c>
-      <c r="J1" s="3">
+      <c r="J1" s="13">
         <v>2029</v>
       </c>
-      <c r="K1" s="3">
+      <c r="K1" s="13">
         <v>2030</v>
       </c>
-      <c r="L1" s="3">
+      <c r="L1" s="13">
         <v>2031</v>
       </c>
-      <c r="M1" s="3">
+      <c r="M1" s="13">
         <v>2032</v>
       </c>
-      <c r="N1" s="3">
+      <c r="N1" s="13">
         <v>2033</v>
       </c>
-      <c r="O1" s="3">
+      <c r="O1" s="13">
         <v>2034</v>
       </c>
-      <c r="P1" s="3">
+      <c r="P1" s="13">
         <v>2035</v>
       </c>
-      <c r="Q1" s="3">
+      <c r="Q1" s="13">
         <v>2036</v>
       </c>
-      <c r="R1" s="3">
+      <c r="R1" s="13">
         <v>2037</v>
       </c>
-      <c r="S1" s="3">
+      <c r="S1" s="13">
         <v>2038</v>
       </c>
-      <c r="T1" s="3">
+      <c r="T1" s="13">
         <v>2039</v>
       </c>
-      <c r="U1" s="3">
+      <c r="U1" s="13">
         <v>2040</v>
       </c>
-      <c r="V1" s="3">
+      <c r="V1" s="13">
         <v>2041</v>
       </c>
-      <c r="W1" s="3">
+      <c r="W1" s="13">
         <v>2042</v>
       </c>
-      <c r="X1" s="3">
+      <c r="X1" s="13">
         <v>2043</v>
       </c>
-      <c r="Y1" s="3">
+      <c r="Y1" s="13">
         <v>2044</v>
       </c>
-      <c r="Z1" s="3">
+      <c r="Z1" s="13">
         <v>2045</v>
       </c>
-      <c r="AA1" s="3">
+      <c r="AA1" s="13">
         <v>2046</v>
       </c>
-      <c r="AB1" s="3">
+      <c r="AB1" s="13">
         <v>2047</v>
       </c>
-      <c r="AC1" s="3">
+      <c r="AC1" s="13">
         <v>2048</v>
       </c>
-      <c r="AD1" s="3">
+      <c r="AD1" s="13">
         <v>2049</v>
       </c>
-      <c r="AE1" s="3">
+      <c r="AE1" s="13">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="2" spans="1:31">
+      <c r="A2" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="12">
         <f>장래가구추계!D2</f>
         <v>21272581</v>
       </c>
-      <c r="C2" s="13">
+      <c r="C2" s="12">
         <f>장래가구추계!E2</f>
         <v>21663978</v>
       </c>
-      <c r="D2" s="13">
+      <c r="D2" s="12">
         <f>장래가구추계!F2</f>
         <v>21970523</v>
       </c>
-      <c r="E2" s="13">
+      <c r="E2" s="12">
         <f>장래가구추계!G2</f>
         <v>22179969</v>
       </c>
-      <c r="F2" s="13">
+      <c r="F2" s="12">
         <f>장래가구추계!H2</f>
         <v>22388821</v>
       </c>
-      <c r="G2" s="13">
+      <c r="G2" s="12">
         <f>장래가구추계!I2</f>
         <v>22597677</v>
       </c>
-      <c r="H2" s="13">
+      <c r="H2" s="12">
         <f>장래가구추계!J2</f>
         <v>22806529</v>
       </c>
-      <c r="I2" s="13">
+      <c r="I2" s="12">
         <f>장래가구추계!K2</f>
         <v>23000187</v>
       </c>
-      <c r="J2" s="13">
+      <c r="J2" s="12">
         <f>장래가구추계!L2</f>
         <v>23180688</v>
       </c>
-      <c r="K2" s="13">
+      <c r="K2" s="12">
         <f>장래가구추계!M2</f>
         <v>23348528</v>
       </c>
-      <c r="L2" s="13">
+      <c r="L2" s="12">
         <f>장래가구추계!N2</f>
         <v>23506021</v>
       </c>
-      <c r="M2" s="13">
+      <c r="M2" s="12">
         <f>장래가구추계!O2</f>
         <v>23651567</v>
       </c>
-      <c r="N2" s="13">
+      <c r="N2" s="12">
         <f>장래가구추계!P2</f>
         <v>23786407</v>
       </c>
-      <c r="O2" s="13">
+      <c r="O2" s="12">
         <f>장래가구추계!Q2</f>
         <v>23908631</v>
       </c>
-      <c r="P2" s="13">
+      <c r="P2" s="12">
         <f>장래가구추계!R2</f>
         <v>24019901</v>
       </c>
-      <c r="Q2" s="13">
+      <c r="Q2" s="12">
         <f>장래가구추계!S2</f>
         <v>24119593</v>
       </c>
-      <c r="R2" s="13">
+      <c r="R2" s="12">
         <f>장래가구추계!T2</f>
         <v>24204775</v>
       </c>
-      <c r="S2" s="13">
+      <c r="S2" s="12">
         <f>장래가구추계!U2</f>
         <v>24273745</v>
       </c>
-      <c r="T2" s="13">
+      <c r="T2" s="12">
         <f>장래가구추계!V2</f>
         <v>24325345</v>
       </c>
-      <c r="U2" s="13">
+      <c r="U2" s="12">
         <f>장래가구추계!W2</f>
         <v>24358286</v>
       </c>
-      <c r="V2" s="13">
+      <c r="V2" s="12">
         <f>장래가구추계!X2</f>
         <v>24371931</v>
       </c>
-      <c r="W2" s="13">
+      <c r="W2" s="12">
         <f>장래가구추계!Y2</f>
         <v>24365630</v>
       </c>
-      <c r="X2" s="13">
+      <c r="X2" s="12">
         <f>장래가구추계!Z2</f>
         <v>24338645</v>
       </c>
-      <c r="Y2" s="13">
+      <c r="Y2" s="12">
         <f>장래가구추계!AA2</f>
         <v>24290684</v>
       </c>
-      <c r="Z2" s="13">
+      <c r="Z2" s="12">
         <f>장래가구추계!AB2</f>
         <v>24221145</v>
       </c>
-      <c r="AA2" s="13">
+      <c r="AA2" s="12">
         <f>장래가구추계!AC2</f>
         <v>24131623</v>
       </c>
-      <c r="AB2" s="13">
+      <c r="AB2" s="12">
         <f>장래가구추계!AD2</f>
         <v>24023713</v>
       </c>
-      <c r="AC2" s="13">
+      <c r="AC2" s="12">
         <f>장래가구추계!AE2</f>
         <v>23899146</v>
       </c>
-      <c r="AD2" s="13">
+      <c r="AD2" s="12">
         <f>장래가구추계!AF2</f>
         <v>23760443</v>
       </c>
-      <c r="AE2" s="13">
+      <c r="AE2" s="12">
         <f>장래가구추계!AG2</f>
         <v>23609533</v>
       </c>

</xml_diff>